<commit_message>
Fixed BaseTest getDriver and enabled headless mode
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="15">
   <si>
     <t>Username</t>
   </si>
@@ -55,6 +55,12 @@
   </si>
   <si>
     <t>TestPass@130028</t>
+  </si>
+  <si>
+    <t>QAUser0617205046</t>
+  </si>
+  <si>
+    <t>TestPass@205046</t>
   </si>
 </sst>
 </file>
@@ -395,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
@@ -458,6 +464,26 @@
         <v>10</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Cleared stale test data from Excel file
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData.xlsx
+++ b/src/test/resources/TestData.xlsx
@@ -3,71 +3,20 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{C73D7B40-F954-4406-8CAE-8868518F526C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{D87F5F46-9326-41CC-8449-2CA420CDBDCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Login data" sheetId="7" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="8" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
   <oleSize ref="A1:M8"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="15">
-  <si>
-    <t>Username</t>
-  </si>
-  <si>
-    <t>Password</t>
-  </si>
-  <si>
-    <t>TransferAmount</t>
-  </si>
-  <si>
-    <t>SearchAmount</t>
-  </si>
-  <si>
-    <t>SearchDate</t>
-  </si>
-  <si>
-    <t>SearchTransactionID</t>
-  </si>
-  <si>
-    <t>QAUser0617125445</t>
-  </si>
-  <si>
-    <t>TestPass@125445</t>
-  </si>
-  <si>
-    <t>50</t>
-  </si>
-  <si>
-    <t>06-17-2026</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>QAUser0617130028</t>
-  </si>
-  <si>
-    <t>TestPass@130028</t>
-  </si>
-  <si>
-    <t>QAUser0617205046</t>
-  </si>
-  <si>
-    <t>TestPass@205046</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -400,91 +349,10 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3FF500F-6564-4FFA-AEC6-0879ED37B975}">
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" t="s" s="0">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s" s="0">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s" s="0">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s" s="0">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s" s="0">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" t="s" s="0">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s" s="0">
-        <v>7</v>
-      </c>
-      <c r="C2" t="s" s="0">
-        <v>8</v>
-      </c>
-      <c r="D2" t="s" s="0">
-        <v>8</v>
-      </c>
-      <c r="E2" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="F2" t="s" s="0">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s" s="0">
-        <v>11</v>
-      </c>
-      <c r="B3" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="C3" t="s" s="0">
-        <v>8</v>
-      </c>
-      <c r="D3" t="s" s="0">
-        <v>8</v>
-      </c>
-      <c r="E3" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="F3" t="s" s="0">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s" s="0">
-        <v>13</v>
-      </c>
-      <c r="B4" t="s" s="0">
-        <v>14</v>
-      </c>
-      <c r="C4" t="s" s="0">
-        <v>8</v>
-      </c>
-      <c r="D4" t="s" s="0">
-        <v>8</v>
-      </c>
-      <c r="E4" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="F4" t="s" s="0">
-        <v>10</v>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>